<commit_message>
Snart klar til første kamp
</commit_message>
<xml_diff>
--- a/xlsx/world_cup_2026_hs.xlsx
+++ b/xlsx/world_cup_2026_hs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uio-my.sharepoint.com/personal/haavas_uio_no/Documents/Skrivebord/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haavas\git\VM2026\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="8_{17689BCD-4937-43F7-8D50-56541C7E2778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F3BA07A-23FE-45E1-A794-55DF187BBE90}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D85A98-860D-46C2-942A-54BB8FE7CEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47453,13 +47453,13 @@
         <v>France</v>
       </c>
       <c r="CO37" s="57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CP37" s="59"/>
       <c r="CQ37" s="21"/>
       <c r="CR37" s="107">
         <f>IF(OR(CO37="",CO38="",AND(CP37="",CP38&lt;&gt;""),AND(CP38="",CP37&lt;&gt;""),AND(CQ37="",CQ38&lt;&gt;""),AND(CQ38="",CQ37&lt;&gt;"")),"",CO37*1000+CP37*10+CQ37)</f>
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="38" spans="1:96" x14ac:dyDescent="0.35">
@@ -47726,13 +47726,13 @@
         <v>England</v>
       </c>
       <c r="CO38" s="58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CP38" s="60"/>
       <c r="CQ38" s="23"/>
       <c r="CR38" s="107">
         <f>IF(CR37="","",CO38*1000+CP38*10+CQ38)</f>
-        <v>1000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="39" spans="1:96" x14ac:dyDescent="0.35">
@@ -54551,7 +54551,7 @@
       <c r="CJ68" s="163"/>
       <c r="CK68" s="153" t="str">
         <f>IF(CR37&gt;CR38,CN37,IF(CR37&lt;CR38,CN38,""))</f>
-        <v>France</v>
+        <v>England</v>
       </c>
       <c r="CL68" s="153"/>
       <c r="CM68" s="153"/>

</xml_diff>